<commit_message>
Normalize XLSX dates as ISO text
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/import/xlsx-dates-and-types.xlsx
+++ b/tests/fixtures/import/xlsx-dates-and-types.xlsx
@@ -34,7 +34,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -67,7 +67,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>